<commit_message>
migration data set completed
</commit_message>
<xml_diff>
--- a/migration/tables.xlsx
+++ b/migration/tables.xlsx
@@ -5,32 +5,34 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\migration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\082_083\ward1\migration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91E1768E-6645-4FF9-85FA-45983B8FEBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4AA62B8-92AD-4C8E-8193-AF02823E51C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="10" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="12" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reasons for leaving origin" sheetId="1" r:id="rId1"/>
-    <sheet name="Distribution of Households" sheetId="2" r:id="rId2"/>
-    <sheet name="Satisfaction" sheetId="3" r:id="rId3"/>
-    <sheet name="Datewise migrants no." sheetId="4" r:id="rId4"/>
-    <sheet name="Literacy status" sheetId="6" r:id="rId5"/>
-    <sheet name="Ethnicity" sheetId="5" r:id="rId6"/>
-    <sheet name="Religion" sheetId="7" r:id="rId7"/>
-    <sheet name="Land holdings" sheetId="8" r:id="rId8"/>
-    <sheet name="Water source" sheetId="9" r:id="rId9"/>
-    <sheet name="5yrs age group" sheetId="10" r:id="rId10"/>
-    <sheet name="Marrital status" sheetId="11" r:id="rId11"/>
-    <sheet name="Family size" sheetId="12" r:id="rId12"/>
-    <sheet name="dependency ratio" sheetId="13" r:id="rId13"/>
-    <sheet name="Leaving origin" sheetId="14" r:id="rId14"/>
-    <sheet name="Place of Origin" sheetId="15" r:id="rId15"/>
+    <sheet name="Consequence for Local" sheetId="16" r:id="rId2"/>
+    <sheet name="Distribution of Households" sheetId="2" r:id="rId3"/>
+    <sheet name="Satisfaction" sheetId="3" r:id="rId4"/>
+    <sheet name="Datewise migrants no." sheetId="4" r:id="rId5"/>
+    <sheet name="Literacy status" sheetId="6" r:id="rId6"/>
+    <sheet name="Ethnicity" sheetId="5" r:id="rId7"/>
+    <sheet name="Religion" sheetId="7" r:id="rId8"/>
+    <sheet name="Land holdings" sheetId="8" r:id="rId9"/>
+    <sheet name="Water source" sheetId="9" r:id="rId10"/>
+    <sheet name="5yrs age group" sheetId="10" r:id="rId11"/>
+    <sheet name="Marrital status" sheetId="11" r:id="rId12"/>
+    <sheet name="Family size" sheetId="12" r:id="rId13"/>
+    <sheet name="dependency ratio" sheetId="13" r:id="rId14"/>
+    <sheet name="Leaving origin" sheetId="14" state="hidden" r:id="rId15"/>
+    <sheet name="Reason leaving origin" sheetId="17" r:id="rId16"/>
+    <sheet name="Place of Origin" sheetId="15" r:id="rId17"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId16"/>
+    <externalReference r:id="rId18"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="116">
   <si>
     <t>2. Table No. 5.1.1: Distribution of Reasons for Leaving Place of Origin</t>
   </si>
@@ -338,15 +340,6 @@
     <t>Political Instability</t>
   </si>
   <si>
-    <t>Country</t>
-  </si>
-  <si>
-    <t>District</t>
-  </si>
-  <si>
-    <t>VDC/Municipality</t>
-  </si>
-  <si>
     <t>Same palika</t>
   </si>
   <si>
@@ -387,6 +380,27 @@
   </si>
   <si>
     <t>Not stated</t>
+  </si>
+  <si>
+    <t>Reason for leaving</t>
+  </si>
+  <si>
+    <t>Government job</t>
+  </si>
+  <si>
+    <t>Limited market</t>
+  </si>
+  <si>
+    <t>Limited arable land</t>
+  </si>
+  <si>
+    <t>Limited job opportunity</t>
+  </si>
+  <si>
+    <t>Limited infrastructure</t>
+  </si>
+  <si>
+    <t>Victim of conflict</t>
   </si>
 </sst>
 </file>
@@ -2682,6 +2696,800 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:pattFill prst="pct5">
+              <a:fgClr>
+                <a:schemeClr val="dk1"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:schemeClr val="bg1"/>
+              </a:bgClr>
+            </a:pattFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Reason leaving origin'!$E$2:$E$7</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Limited market</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Limited arable land</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Limited job opportunity</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Limited infrastructure</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Government job</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Victim of conflict</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Reason leaving origin'!$F$2:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>20.224719101123593</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7.8651685393258424</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>26.966292134831459</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34.831460674157306</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.6179775280898872</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.4943820224719104</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9921-45F9-B1D2-DD6AEB167957}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="80"/>
+        <c:overlap val="25"/>
+        <c:axId val="1141911823"/>
+        <c:axId val="1746210975"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1141911823"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Reasons for leaving</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> origin</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                </a:endParaRPr>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="15875" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="20" normalizeH="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1746210975"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1746210975"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="5000"/>
+                  <a:lumOff val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Percentage</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> (%)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                </a:endParaRPr>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="20" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1141911823"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="lt1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:view3D>
+      <c:rotX val="30"/>
+      <c:rotY val="0"/>
+      <c:depthPercent val="100"/>
+      <c:rAngAx val="0"/>
+    </c:view3D>
+    <c:floor>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:floor>
+    <c:sideWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:sideWall>
+    <c:backWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:backWall>
+    <c:plotArea>
+      <c:layout/>
+      <c:pie3DChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="diagBrick">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="tx1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-CB81-4E4F-BFFF-ECBBBD34CE17}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="ltUpDiag">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="tx1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-CB81-4E4F-BFFF-ECBBBD34CE17}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="pct5">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="tx1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-CB81-4E4F-BFFF-ECBBBD34CE17}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:gradFill>
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="5000"/>
+                      <a:lumOff val="95000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="74000">
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="45000"/>
+                      <a:lumOff val="55000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="83000">
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="45000"/>
+                      <a:lumOff val="55000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="30000"/>
+                      <a:lumOff val="70000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000" scaled="1"/>
+              </a:gradFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="bestFit"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:round/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Place of Origin'!$E$3:$E$5</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Same palika</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Other palika of same district</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Other district</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Place of Origin'!$F$3:$F$5</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>5.6179775280898872</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>21.348314606741571</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>73.033707865168537</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-CB81-4E4F-BFFF-ECBBBD34CE17}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="bestFit"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+      </c:pie3DChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
@@ -4093,10 +4901,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>62</c:v>
+                  <c:v>79</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
@@ -6249,6 +7057,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors14.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors15.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -9132,6 +10020,1017 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style14.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="215">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="15875" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200" cap="none" spc="20" normalizeH="0" baseline="0"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="bg1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="50000"/>
+          <a:lumOff val="50000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="70000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="70000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:alpha val="70000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr">
+          <a:alpha val="70000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200" baseline="0"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="major">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="0" i="0" kern="1200" cap="none" spc="50" normalizeH="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="15875" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200" spc="20" baseline="0"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style15.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="262">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
   <cs:axisTitle>
@@ -13225,6 +15124,88 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>99060</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>156210</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{83793400-371C-D104-249D-A0000A5DB4C3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>426720</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>472440</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6FEF239-81DD-10B3-DE30-F9B5AC44858E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -14012,15 +15993,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -14033,7 +16014,7 @@
       <c r="H1" s="17"/>
       <c r="I1" s="17"/>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
@@ -14046,7 +16027,7 @@
       <c r="H2" s="18"/>
       <c r="I2" s="18"/>
     </row>
-    <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -14057,7 +16038,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -14068,7 +16049,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
@@ -14079,7 +16060,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
@@ -14090,7 +16071,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -14101,7 +16082,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
@@ -14112,7 +16093,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -14123,7 +16104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>11</v>
       </c>
@@ -14134,7 +16115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>12</v>
       </c>
@@ -14156,19 +16137,116 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A37B388-6521-440D-9FFB-5546F102E9EC}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="9">
+        <v>48</v>
+      </c>
+      <c r="C2" s="11">
+        <f>B2/B5*100</f>
+        <v>53.932584269662918</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G2" s="11">
+        <f>C2</f>
+        <v>53.932584269662918</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="9">
+        <v>35</v>
+      </c>
+      <c r="C3" s="11">
+        <f>B3/B5*100</f>
+        <v>39.325842696629216</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="11">
+        <f t="shared" ref="G3:G4" si="0">C3</f>
+        <v>39.325842696629216</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="9">
+        <v>6</v>
+      </c>
+      <c r="C4" s="11">
+        <f>B4/B5*100</f>
+        <v>6.7415730337078648</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="11">
+        <f t="shared" si="0"/>
+        <v>6.7415730337078648</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="9">
+        <f>SUM(B2:B4)</f>
+        <v>89</v>
+      </c>
+      <c r="C5" s="9">
+        <f>SUM(C2:C4)</f>
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4681C5CD-AD1E-47C1-9DD5-E5803D1EB1C3}">
   <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
         <v>72</v>
       </c>
@@ -14185,7 +16263,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="20"/>
       <c r="B2" s="9" t="s">
         <v>36</v>
@@ -14202,7 +16280,7 @@
       <c r="F2" s="19"/>
       <c r="G2" s="19"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>57</v>
       </c>
@@ -14232,7 +16310,7 @@
         <v>2.8769707586578628</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
         <v>58</v>
       </c>
@@ -14262,7 +16340,7 @@
         <v>3.1532138525805147</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
         <v>59</v>
       </c>
@@ -14292,7 +16370,7 @@
         <v>7.2210618515024931</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
         <v>60</v>
       </c>
@@ -14322,7 +16400,7 @@
         <v>4.9824821452634414</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
         <v>61</v>
       </c>
@@ -14352,7 +16430,7 @@
         <v>9.4882765125993807</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
         <v>62</v>
       </c>
@@ -14382,7 +16460,7 @@
         <v>8.7168171405470964</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
         <v>63</v>
       </c>
@@ -14412,7 +16490,7 @@
         <v>10.431545613798679</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
         <v>64</v>
       </c>
@@ -14442,7 +16520,7 @@
         <v>8.497843956340116</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
         <v>65</v>
       </c>
@@ -14472,7 +16550,7 @@
         <v>9.7173561514620665</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
         <v>66</v>
       </c>
@@ -14502,7 +16580,7 @@
         <v>7.6876431747742888</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
         <v>67</v>
       </c>
@@ -14532,7 +16610,7 @@
         <v>8.8027220051206037</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>68</v>
       </c>
@@ -14562,7 +16640,7 @@
         <v>8.0784260881282837</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
         <v>69</v>
       </c>
@@ -14592,7 +16670,7 @@
         <v>3.6770650855679827</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>70</v>
       </c>
@@ -14622,7 +16700,7 @@
         <v>6.6685756636571893</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>12</v>
       </c>
@@ -14660,25 +16738,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5FC4570-8427-483C-9157-77FE223CE978}">
   <dimension ref="A1:O7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.7109375" customWidth="1"/>
-    <col min="13" max="13" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.6640625" customWidth="1"/>
+    <col min="13" max="13" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
         <v>73</v>
       </c>
@@ -14693,7 +16771,7 @@
       </c>
       <c r="G1" s="19"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="20"/>
       <c r="B2" s="21" t="s">
         <v>36</v>
@@ -14712,7 +16790,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="20"/>
       <c r="B3" s="9" t="s">
         <v>74</v>
@@ -14744,7 +16822,7 @@
         <v>34.615384615384613</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>75</v>
       </c>
@@ -14792,7 +16870,7 @@
         <v>65.384615384615387</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>76</v>
       </c>
@@ -14829,7 +16907,7 @@
         <v>62.037037037037038</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -14859,7 +16937,7 @@
       </c>
       <c r="K6" s="13"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="K7" s="13"/>
     </row>
   </sheetData>
@@ -14876,17 +16954,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3986BFF3-A766-496C-9200-083AC941658F}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>82</v>
       </c>
@@ -14897,7 +16975,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>79</v>
       </c>
@@ -14916,7 +16994,7 @@
         <v>77.528089887640448</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>80</v>
       </c>
@@ -14935,7 +17013,7 @@
         <v>16.853932584269664</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>81</v>
       </c>
@@ -14954,7 +17032,7 @@
         <v>5.6179775280898872</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>12</v>
       </c>
@@ -14975,15 +17053,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC3014F1-1703-47D5-A2CD-2B891BFB9566}">
   <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>83</v>
       </c>
@@ -15007,7 +17085,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>84</v>
       </c>
@@ -15037,7 +17115,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>85</v>
       </c>
@@ -15067,7 +17145,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
@@ -15103,20 +17181,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDF745B5-F0A4-4C32-BF38-D8BF1F0ED0B6}">
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>90</v>
       </c>
@@ -15127,114 +17205,114 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>92</v>
       </c>
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>93</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>94</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -15244,133 +17322,281 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E211E5C9-7DF2-4829-BE18-8FD1E5D07B3F}">
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE692314-3B3B-4824-945E-BC96E76CCF72}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
-        <v>15</v>
+        <v>109</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="9">
+        <v>18</v>
+      </c>
+      <c r="C2" s="11">
+        <f>B2/$B$8*100</f>
+        <v>20.224719101123593</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" s="11">
+        <f>C2</f>
+        <v>20.224719101123593</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="9">
+        <v>7</v>
+      </c>
+      <c r="C3" s="11">
+        <f t="shared" ref="C3:C8" si="0">B3/$B$8*100</f>
+        <v>7.8651685393258424</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="F3" s="11">
+        <f t="shared" ref="F3:F7" si="1">C3</f>
+        <v>7.8651685393258424</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="9">
+        <v>24</v>
+      </c>
+      <c r="C4" s="11">
+        <f t="shared" si="0"/>
+        <v>26.966292134831459</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F4" s="11">
+        <f t="shared" si="1"/>
+        <v>26.966292134831459</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" s="9">
+        <v>31</v>
+      </c>
+      <c r="C5" s="11">
+        <f t="shared" si="0"/>
+        <v>34.831460674157306</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="F5" s="11">
+        <f t="shared" si="1"/>
+        <v>34.831460674157306</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" s="9">
+        <v>5</v>
+      </c>
+      <c r="C6" s="11">
+        <f t="shared" si="0"/>
+        <v>5.6179775280898872</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="F6" s="11">
+        <f t="shared" si="1"/>
+        <v>5.6179775280898872</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7" s="9">
+        <v>4</v>
+      </c>
+      <c r="C7" s="11">
+        <f t="shared" si="0"/>
+        <v>4.4943820224719104</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="F7" s="11">
+        <f t="shared" si="1"/>
+        <v>4.4943820224719104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="9">
+        <f>SUM(B2:B7)</f>
+        <v>89</v>
+      </c>
+      <c r="C8" s="11">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E211E5C9-7DF2-4829-BE18-8FD1E5D07B3F}">
+  <dimension ref="A2:F6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
+      <c r="B3" s="9">
+        <v>5</v>
+      </c>
+      <c r="C3" s="11">
+        <f>B3/$B$6*100</f>
+        <v>5.6179775280898872</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F3" s="11">
+        <f>C3</f>
+        <v>5.6179775280898872</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
+      <c r="B4" s="9">
+        <f>24-B3</f>
+        <v>19</v>
+      </c>
+      <c r="C4" s="11">
+        <f t="shared" ref="C4:C6" si="0">B4/$B$6*100</f>
+        <v>21.348314606741571</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" s="11">
+        <f t="shared" ref="F4:F5" si="1">C4</f>
+        <v>21.348314606741571</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="B8" s="9">
-        <v>5</v>
-      </c>
-      <c r="C8" s="11">
-        <f>B8/$B$11*100</f>
-        <v>5.6179775280898872</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="B9" s="9">
-        <f>24-B8</f>
-        <v>19</v>
-      </c>
-      <c r="C9" s="11">
-        <f t="shared" ref="C9:C11" si="0">B9/$B$11*100</f>
-        <v>21.348314606741571</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="B10" s="9">
+      <c r="B5" s="9">
         <v>65</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C5" s="11">
         <f t="shared" si="0"/>
         <v>73.033707865168537</v>
       </c>
+      <c r="E5" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F5" s="11">
+        <f t="shared" si="1"/>
+        <v>73.033707865168537</v>
+      </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="9">
-        <f>SUM(B8:B10)</f>
+      <c r="B6" s="9">
+        <f>SUM(B3:B5)</f>
         <v>89</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C6" s="11">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A66E6E1-0788-40AD-8F74-B033FAAE0A65}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>13</v>
       </c>
@@ -15386,7 +17612,7 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="18" t="s">
         <v>14</v>
       </c>
@@ -15402,7 +17628,7 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
@@ -15413,7 +17639,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
@@ -15424,7 +17650,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>17</v>
       </c>
@@ -15435,7 +17661,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
@@ -15446,7 +17672,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -15467,19 +17693,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>19</v>
       </c>
@@ -15494,7 +17720,7 @@
       <c r="J1" s="17"/>
       <c r="K1" s="17"/>
     </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -15509,7 +17735,7 @@
       <c r="J2" s="18"/>
       <c r="K2" s="18"/>
     </row>
-    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
@@ -15520,7 +17746,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -15528,10 +17754,10 @@
         <v>0.76500000000000001</v>
       </c>
       <c r="C4" s="6">
-        <v>62</v>
+        <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>23</v>
       </c>
@@ -15539,10 +17765,10 @@
         <v>0.21</v>
       </c>
       <c r="C5" s="6">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>24</v>
       </c>
@@ -15553,7 +17779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -15561,7 +17787,8 @@
         <v>1</v>
       </c>
       <c r="C7" s="6">
-        <v>81</v>
+        <f>SUM(C4:C6)</f>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -15574,15 +17801,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>25</v>
       </c>
@@ -15590,7 +17817,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="9">
         <v>2083</v>
       </c>
@@ -15598,7 +17825,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="9">
         <v>2082</v>
       </c>
@@ -15606,7 +17833,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
         <v>2081</v>
       </c>
@@ -15614,7 +17841,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
         <v>2080</v>
       </c>
@@ -15622,7 +17849,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="9">
         <v>2079</v>
       </c>
@@ -15630,7 +17857,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="9">
         <v>2078</v>
       </c>
@@ -15638,7 +17865,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
         <v>2077</v>
       </c>
@@ -15646,7 +17873,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
         <v>2076</v>
       </c>
@@ -15654,7 +17881,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
         <v>2075</v>
       </c>
@@ -15662,7 +17889,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
         <v>2074</v>
       </c>
@@ -15670,7 +17897,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>12</v>
       </c>
@@ -15685,12 +17912,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
         <v>33</v>
       </c>
@@ -15705,7 +17932,7 @@
       </c>
       <c r="G1" s="20"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="20"/>
       <c r="B2" s="19" t="s">
         <v>36</v>
@@ -15718,7 +17945,7 @@
       <c r="F2" s="20"/>
       <c r="G2" s="20"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="20"/>
       <c r="B3" s="10" t="s">
         <v>37</v>
@@ -15745,7 +17972,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>38</v>
       </c>
@@ -15781,7 +18008,7 @@
         <v>66.875</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>39</v>
       </c>
@@ -15817,7 +18044,7 @@
         <v>33.125</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -15859,15 +18086,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>27</v>
       </c>
@@ -15878,215 +18105,96 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>30</v>
       </c>
       <c r="B2" s="9">
-        <f ca="1">'[1]for graph'!$I$4</f>
+        <f>'[1]for graph'!$I$4</f>
         <v>28</v>
       </c>
       <c r="C2" s="11">
-        <f ca="1">B2/B6*100</f>
+        <f>B2/B6*100</f>
         <v>31.460674157303369</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>30</v>
       </c>
       <c r="G2" s="11">
-        <f ca="1">C2</f>
+        <f>C2</f>
         <v>31.460674157303369</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="9">
-        <f ca="1">'[1]for graph'!$I$3</f>
+        <f>'[1]for graph'!$I$3</f>
         <v>32</v>
       </c>
       <c r="C3" s="11">
-        <f ca="1">B3/B6*100</f>
+        <f>B3/B6*100</f>
         <v>35.955056179775283</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>31</v>
       </c>
       <c r="G3" s="11">
-        <f t="shared" ref="G3:G5" ca="1" si="0">C3</f>
+        <f t="shared" ref="G3:G5" si="0">C3</f>
         <v>35.955056179775283</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
       <c r="B4" s="9">
-        <f ca="1">'[1]for graph'!$I$14</f>
+        <f>'[1]for graph'!$I$14</f>
         <v>23</v>
       </c>
       <c r="C4" s="11">
-        <f ca="1">B4/B6*100</f>
+        <f>B4/B6*100</f>
         <v>25.842696629213485</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>40</v>
       </c>
       <c r="G4" s="11">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>25.842696629213485</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>41</v>
       </c>
       <c r="B5" s="9">
-        <f ca="1">'[1]for graph'!$I$6</f>
+        <f>'[1]for graph'!$I$6</f>
         <v>6</v>
       </c>
       <c r="C5" s="11">
-        <f ca="1">B5/B6*100</f>
+        <f>B5/B6*100</f>
         <v>6.7415730337078648</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>41</v>
       </c>
       <c r="G5" s="11">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>6.7415730337078648</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="9">
-        <f ca="1">SUM(B2:B5)</f>
+        <f>SUM(B2:B5)</f>
         <v>89</v>
       </c>
       <c r="C6" s="9">
-        <f ca="1">SUM(C2:C5)</f>
-        <v>100.00000000000001</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17375082-251D-4B38-966E-F88F9E772705}">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2" s="9">
-        <f ca="1">'[1]for graph'!$K$3</f>
-        <v>60</v>
-      </c>
-      <c r="C2" s="11">
-        <f ca="1">B2/B6*100</f>
-        <v>67.415730337078656</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="G2" s="11">
-        <f ca="1">C2</f>
-        <v>67.415730337078656</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="9">
-        <f ca="1">'[1]for graph'!$K$14</f>
-        <v>23</v>
-      </c>
-      <c r="C3" s="11">
-        <f ca="1">B3/B6*100</f>
-        <v>25.842696629213485</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="11">
-        <f ca="1">C3</f>
-        <v>25.842696629213485</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="9">
-        <v>0</v>
-      </c>
-      <c r="C4" s="11">
-        <f ca="1">B4/B6*100</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="11">
-        <f ca="1">C4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="9">
-        <f ca="1">'[1]for graph'!$K$6</f>
-        <v>6</v>
-      </c>
-      <c r="C5" s="11">
-        <f ca="1">B5/B6*100</f>
-        <v>6.7415730337078648</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="G5" s="11">
-        <f ca="1">C5</f>
-        <v>6.7415730337078648</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="9">
-        <f ca="1">SUM(B2:B5)</f>
-        <v>89</v>
-      </c>
-      <c r="C6" s="9">
-        <f ca="1">SUM(C2:C5)</f>
+        <f>SUM(C2:C5)</f>
         <v>100.00000000000001</v>
       </c>
     </row>
@@ -16098,16 +18206,135 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17375082-251D-4B38-966E-F88F9E772705}">
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="9">
+        <f>'[1]for graph'!$K$3</f>
+        <v>60</v>
+      </c>
+      <c r="C2" s="11">
+        <f>B2/B6*100</f>
+        <v>67.415730337078656</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="11">
+        <f>C2</f>
+        <v>67.415730337078656</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="9">
+        <f>'[1]for graph'!$K$14</f>
+        <v>23</v>
+      </c>
+      <c r="C3" s="11">
+        <f>B3/B6*100</f>
+        <v>25.842696629213485</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="11">
+        <f>C3</f>
+        <v>25.842696629213485</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="9">
+        <v>0</v>
+      </c>
+      <c r="C4" s="11">
+        <f>B4/B6*100</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="11">
+        <f>C4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="9">
+        <f>'[1]for graph'!$K$6</f>
+        <v>6</v>
+      </c>
+      <c r="C5" s="11">
+        <f>B5/B6*100</f>
+        <v>6.7415730337078648</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="11">
+        <f>C5</f>
+        <v>6.7415730337078648</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="9">
+        <f>SUM(B2:B5)</f>
+        <v>89</v>
+      </c>
+      <c r="C6" s="9">
+        <f>SUM(C2:C5)</f>
+        <v>100.00000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313C3968-0C2C-495D-B103-63BB836806C3}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>47</v>
       </c>
@@ -16118,7 +18345,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>49</v>
       </c>
@@ -16131,7 +18358,7 @@
         <v>17.977528089887642</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>50</v>
       </c>
@@ -16144,7 +18371,7 @@
         <v>69.662921348314612</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>51</v>
       </c>
@@ -16156,7 +18383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>52</v>
       </c>
@@ -16168,7 +18395,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>32</v>
       </c>
@@ -16180,7 +18407,7 @@
         <v>12.359550561797752</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
         <v>12</v>
       </c>
@@ -16197,101 +18424,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A37B388-6521-440D-9FFB-5546F102E9EC}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="9">
-        <v>48</v>
-      </c>
-      <c r="C2" s="11">
-        <f>B2/B5*100</f>
-        <v>53.932584269662918</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="G2" s="11">
-        <f>C2</f>
-        <v>53.932584269662918</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B3" s="9">
-        <v>35</v>
-      </c>
-      <c r="C3" s="11">
-        <f>B3/B5*100</f>
-        <v>39.325842696629216</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="G3" s="11">
-        <f t="shared" ref="G3:G4" si="0">C3</f>
-        <v>39.325842696629216</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="9">
-        <v>6</v>
-      </c>
-      <c r="C4" s="11">
-        <f>B4/B5*100</f>
-        <v>6.7415730337078648</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" s="11">
-        <f t="shared" si="0"/>
-        <v>6.7415730337078648</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="9">
-        <f>SUM(B2:B4)</f>
-        <v>89</v>
-      </c>
-      <c r="C5" s="9">
-        <f>SUM(C2:C4)</f>
-        <v>100</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
thesis all correction made
</commit_message>
<xml_diff>
--- a/migration/tables.xlsx
+++ b/migration/tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\migration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\082_083\ward1\migration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED59ED29-146D-4349-A008-9240342B8810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56228FFE-3E59-4064-8854-B12E01CAF88D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" firstSheet="21" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3168" yWindow="876" windowWidth="17280" windowHeight="11256" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reasons for leaving origin" sheetId="1" state="hidden" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="171">
   <si>
     <t>2. Table No. 5.1.1: Distribution of Reasons for Leaving Place of Origin</t>
   </si>
@@ -565,6 +565,15 @@
   <si>
     <t>Go to another place</t>
   </si>
+  <si>
+    <t>Male No.</t>
+  </si>
+  <si>
+    <t>Female No.</t>
+  </si>
+  <si>
+    <t>Total No.</t>
+  </si>
 </sst>
 </file>
 
@@ -710,7 +719,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -780,7 +789,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -20816,15 +20824,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -20837,7 +20845,7 @@
       <c r="H1" s="24"/>
       <c r="I1" s="24"/>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
@@ -20850,7 +20858,7 @@
       <c r="H2" s="25"/>
       <c r="I2" s="25"/>
     </row>
-    <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -20861,7 +20869,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -20872,7 +20880,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
@@ -20883,7 +20891,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
@@ -20894,7 +20902,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -20905,7 +20913,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
@@ -20916,7 +20924,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -20927,7 +20935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>11</v>
       </c>
@@ -20938,7 +20946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>12</v>
       </c>
@@ -20961,24 +20969,24 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5FC4570-8427-483C-9157-77FE223CE978}">
-  <dimension ref="A1:O7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.7109375" customWidth="1"/>
-    <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.6640625" customWidth="1"/>
+    <col min="13" max="13" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>73</v>
       </c>
@@ -20993,7 +21001,7 @@
       </c>
       <c r="G1" s="26"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="27"/>
       <c r="B2" s="28" t="s">
         <v>36</v>
@@ -21012,7 +21020,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="27"/>
       <c r="B3" s="9" t="s">
         <v>74</v>
@@ -21044,7 +21052,7 @@
         <v>34.615384615384613</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>75</v>
       </c>
@@ -21090,7 +21098,7 @@
         <v>65.384615384615387</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>76</v>
       </c>
@@ -21125,7 +21133,7 @@
         <v>62.037037037037038</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -21155,8 +21163,114 @@
       </c>
       <c r="K6" s="13"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="K7" s="13"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" s="9">
+        <v>69</v>
+      </c>
+      <c r="C31" s="11">
+        <f>B31/$B$6*100</f>
+        <v>41.071428571428569</v>
+      </c>
+      <c r="D31" s="9">
+        <v>54</v>
+      </c>
+      <c r="E31" s="11">
+        <f>D31/$D$6*100</f>
+        <v>34.615384615384613</v>
+      </c>
+      <c r="F31" s="9">
+        <f>B31+D31</f>
+        <v>123</v>
+      </c>
+      <c r="G31" s="11">
+        <f>F31/$F$6*100</f>
+        <v>37.962962962962962</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B32" s="9">
+        <v>99</v>
+      </c>
+      <c r="C32" s="11">
+        <f t="shared" ref="C32" si="2">B32/$B$6*100</f>
+        <v>58.928571428571431</v>
+      </c>
+      <c r="D32" s="9">
+        <v>102</v>
+      </c>
+      <c r="E32" s="11">
+        <f>D32/$D$6*100</f>
+        <v>65.384615384615387</v>
+      </c>
+      <c r="F32" s="9">
+        <f>B32+D32</f>
+        <v>201</v>
+      </c>
+      <c r="G32" s="11">
+        <f>F32/$F$6*100</f>
+        <v>62.037037037037038</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B33" s="9">
+        <f>SUM(B31:B32)</f>
+        <v>168</v>
+      </c>
+      <c r="C33" s="9">
+        <f t="shared" ref="C33:G33" si="3">SUM(C31:C32)</f>
+        <v>100</v>
+      </c>
+      <c r="D33" s="9">
+        <f t="shared" si="3"/>
+        <v>156</v>
+      </c>
+      <c r="E33" s="9">
+        <f t="shared" si="3"/>
+        <v>100</v>
+      </c>
+      <c r="F33" s="9">
+        <f t="shared" si="3"/>
+        <v>324</v>
+      </c>
+      <c r="G33" s="9">
+        <f t="shared" si="3"/>
+        <v>100</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -21175,14 +21289,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3986BFF3-A766-496C-9200-083AC941658F}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>82</v>
       </c>
@@ -21193,7 +21307,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>79</v>
       </c>
@@ -21212,7 +21326,7 @@
         <v>77.528089887640448</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>80</v>
       </c>
@@ -21231,7 +21345,7 @@
         <v>16.853932584269664</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>81</v>
       </c>
@@ -21250,7 +21364,7 @@
         <v>5.6179775280898872</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>12</v>
       </c>
@@ -21274,12 +21388,12 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC3014F1-1703-47D5-A2CD-2B891BFB9566}">
   <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>83</v>
       </c>
@@ -21303,7 +21417,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>84</v>
       </c>
@@ -21333,7 +21447,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>85</v>
       </c>
@@ -21363,7 +21477,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
@@ -21405,14 +21519,14 @@
     <tabColor rgb="FFC00000"/>
   </sheetPr>
   <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>90</v>
       </c>
@@ -21423,112 +21537,112 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>92</v>
       </c>
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>93</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>94</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>98</v>
       </c>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>99</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>100</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>101</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>102</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>103</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>104</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>105</v>
       </c>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>106</v>
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
         <v>107</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
         <v>108</v>
       </c>
@@ -21543,15 +21657,15 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE692314-3B3B-4824-945E-BC96E76CCF72}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>109</v>
       </c>
@@ -21562,7 +21676,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>111</v>
       </c>
@@ -21581,7 +21695,7 @@
         <v>20.224719101123593</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>112</v>
       </c>
@@ -21600,7 +21714,7 @@
         <v>7.8651685393258424</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>113</v>
       </c>
@@ -21619,7 +21733,7 @@
         <v>26.966292134831459</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>114</v>
       </c>
@@ -21638,7 +21752,7 @@
         <v>34.831460674157306</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>110</v>
       </c>
@@ -21657,7 +21771,7 @@
         <v>5.6179775280898872</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>115</v>
       </c>
@@ -21676,7 +21790,7 @@
         <v>4.4943820224719104</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>12</v>
       </c>
@@ -21698,15 +21812,15 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E211E5C9-7DF2-4829-BE18-8FD1E5D07B3F}">
   <dimension ref="A2:F6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>15</v>
       </c>
@@ -21717,7 +21831,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>95</v>
       </c>
@@ -21736,7 +21850,7 @@
         <v>5.6179775280898872</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>96</v>
       </c>
@@ -21756,7 +21870,7 @@
         <v>21.348314606741571</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>97</v>
       </c>
@@ -21775,7 +21889,7 @@
         <v>73.033707865168537</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>12</v>
       </c>
@@ -21797,16 +21911,16 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E692AE2-61AB-4B81-B25E-1712F371FD92}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>121</v>
       </c>
@@ -21817,7 +21931,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>116</v>
       </c>
@@ -21836,7 +21950,7 @@
         <v>23.595505617977526</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>117</v>
       </c>
@@ -21855,7 +21969,7 @@
         <v>16.853932584269664</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>118</v>
       </c>
@@ -21874,7 +21988,7 @@
         <v>14.606741573033707</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>119</v>
       </c>
@@ -21893,7 +22007,7 @@
         <v>16.853932584269664</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>120</v>
       </c>
@@ -21912,7 +22026,7 @@
         <v>28.08988764044944</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>12</v>
       </c>
@@ -21934,16 +22048,16 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="24" t="s">
         <v>19</v>
       </c>
@@ -21958,7 +22072,7 @@
       <c r="J1" s="24"/>
       <c r="K1" s="24"/>
     </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="25" t="s">
         <v>20</v>
       </c>
@@ -21973,7 +22087,7 @@
       <c r="J2" s="25"/>
       <c r="K2" s="25"/>
     </row>
-    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
@@ -21984,7 +22098,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -21996,7 +22110,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>23</v>
       </c>
@@ -22008,7 +22122,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>24</v>
       </c>
@@ -22020,7 +22134,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -22032,7 +22146,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="5" t="s">
         <v>22</v>
       </c>
@@ -22041,7 +22155,7 @@
         <v>0.88764044943820219</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="5" t="s">
         <v>23</v>
       </c>
@@ -22050,7 +22164,7 @@
         <v>8.98876404494382E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="5" t="s">
         <v>24</v>
       </c>
@@ -22072,16 +22186,16 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E46D432-B2D5-422F-B7B2-6F5D2F13684D}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="32" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>128</v>
       </c>
@@ -22091,10 +22205,8 @@
       <c r="C1" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>123</v>
       </c>
@@ -22102,7 +22214,7 @@
         <v>35</v>
       </c>
       <c r="C2" s="11">
-        <f>B2/$B$7*100</f>
+        <f t="shared" ref="C2:C7" si="0">B2/$B$7*100</f>
         <v>39.325842696629216</v>
       </c>
       <c r="E2" s="9" t="s">
@@ -22113,7 +22225,7 @@
         <v>39.325842696629216</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>124</v>
       </c>
@@ -22121,7 +22233,7 @@
         <v>7</v>
       </c>
       <c r="C3" s="11">
-        <f>B3/$B$7*100</f>
+        <f t="shared" si="0"/>
         <v>7.8651685393258424</v>
       </c>
       <c r="E3" s="9" t="s">
@@ -22132,7 +22244,7 @@
         <v>7.8651685393258424</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>125</v>
       </c>
@@ -22140,7 +22252,7 @@
         <v>14</v>
       </c>
       <c r="C4" s="11">
-        <f>B4/$B$7*100</f>
+        <f t="shared" si="0"/>
         <v>15.730337078651685</v>
       </c>
       <c r="E4" s="9" t="s">
@@ -22151,7 +22263,7 @@
         <v>15.730337078651685</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>126</v>
       </c>
@@ -22159,7 +22271,7 @@
         <v>17</v>
       </c>
       <c r="C5" s="11">
-        <f>B5/$B$7*100</f>
+        <f t="shared" si="0"/>
         <v>19.101123595505616</v>
       </c>
       <c r="E5" s="9" t="s">
@@ -22170,7 +22282,7 @@
         <v>19.101123595505616</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>127</v>
       </c>
@@ -22178,7 +22290,7 @@
         <v>16</v>
       </c>
       <c r="C6" s="11">
-        <f>B6/$B$7*100</f>
+        <f t="shared" si="0"/>
         <v>17.977528089887642</v>
       </c>
       <c r="E6" s="9" t="s">
@@ -22189,7 +22301,7 @@
         <v>17.977528089887642</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>12</v>
       </c>
@@ -22198,7 +22310,7 @@
         <v>89</v>
       </c>
       <c r="C7" s="11">
-        <f>B7/$B$7*100</f>
+        <f t="shared" si="0"/>
         <v>100</v>
       </c>
     </row>
@@ -22211,15 +22323,15 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE47149E-27C5-478E-B746-3FD5C723EB44}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25" style="22" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
         <v>131</v>
       </c>
@@ -22233,7 +22345,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>22</v>
       </c>
@@ -22246,7 +22358,7 @@
       </c>
       <c r="D2" s="10"/>
     </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>23</v>
       </c>
@@ -22261,7 +22373,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>12</v>
       </c>
@@ -22283,15 +22395,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="24" t="s">
         <v>13</v>
       </c>
@@ -22307,7 +22419,7 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="25" t="s">
         <v>14</v>
       </c>
@@ -22323,7 +22435,7 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
@@ -22334,7 +22446,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
@@ -22345,7 +22457,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>17</v>
       </c>
@@ -22356,7 +22468,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
@@ -22367,7 +22479,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -22391,12 +22503,12 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F223E6C1-2682-4AAE-BF49-10A831AC5F17}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>132</v>
       </c>
@@ -22410,7 +22522,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>133</v>
       </c>
@@ -22425,7 +22537,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>136</v>
       </c>
@@ -22440,7 +22552,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>134</v>
       </c>
@@ -22455,7 +22567,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>135</v>
       </c>
@@ -22470,7 +22582,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>132</v>
       </c>
@@ -22484,7 +22596,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>133</v>
       </c>
@@ -22501,7 +22613,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>136</v>
       </c>
@@ -22518,7 +22630,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>134</v>
       </c>
@@ -22535,7 +22647,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>135</v>
       </c>
@@ -22561,16 +22673,16 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D74971AF-D04F-4083-BD95-BE282B014BFD}">
   <dimension ref="A1:E18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
         <v>137</v>
       </c>
@@ -22583,7 +22695,7 @@
       </c>
       <c r="E1" s="26"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="26"/>
       <c r="B2" s="9" t="s">
         <v>139</v>
@@ -22598,7 +22710,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>140</v>
       </c>
@@ -22617,7 +22729,7 @@
         <v>1.1235955056179776</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>141</v>
       </c>
@@ -22636,7 +22748,7 @@
         <v>11.235955056179774</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>142</v>
       </c>
@@ -22655,7 +22767,7 @@
         <v>37.078651685393261</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>143</v>
       </c>
@@ -22674,7 +22786,7 @@
         <v>28.08988764044944</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>144</v>
       </c>
@@ -22693,7 +22805,7 @@
         <v>16.853932584269664</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>145</v>
       </c>
@@ -22712,7 +22824,7 @@
         <v>5.6179775280898872</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>12</v>
       </c>
@@ -22733,7 +22845,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>137</v>
       </c>
@@ -22745,7 +22857,7 @@
       </c>
       <c r="E12" s="10"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>140</v>
       </c>
@@ -22758,7 +22870,7 @@
         <v>1.1235955056179776</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>141</v>
       </c>
@@ -22771,7 +22883,7 @@
         <v>11.235955056179774</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>142</v>
       </c>
@@ -22784,7 +22896,7 @@
         <v>37.078651685393261</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>143</v>
       </c>
@@ -22797,7 +22909,7 @@
         <v>28.08988764044944</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
         <v>144</v>
       </c>
@@ -22810,7 +22922,7 @@
         <v>16.853932584269664</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
         <v>145</v>
       </c>
@@ -22837,14 +22949,14 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{406D7635-71FE-425B-8519-D75FA2CDF8A9}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>136</v>
       </c>
@@ -22855,7 +22967,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>104</v>
       </c>
@@ -22866,7 +22978,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>105</v>
       </c>
@@ -22877,7 +22989,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>103</v>
       </c>
@@ -22888,7 +23000,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>148</v>
       </c>
@@ -22899,7 +23011,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>149</v>
       </c>
@@ -22910,7 +23022,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>110</v>
       </c>
@@ -22921,7 +23033,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>102</v>
       </c>
@@ -22932,7 +23044,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>108</v>
       </c>
@@ -22943,7 +23055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
         <v>12</v>
       </c>
@@ -22956,7 +23068,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>136</v>
       </c>
@@ -22967,7 +23079,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>104</v>
       </c>
@@ -22980,7 +23092,7 @@
         <v>35.955056179775283</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>105</v>
       </c>
@@ -22993,7 +23105,7 @@
         <v>21.348314606741571</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>103</v>
       </c>
@@ -23006,7 +23118,7 @@
         <v>10.112359550561797</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>148</v>
       </c>
@@ -23019,7 +23131,7 @@
         <v>4.4943820224719104</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
         <v>149</v>
       </c>
@@ -23032,7 +23144,7 @@
         <v>19.101123595505616</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
         <v>110</v>
       </c>
@@ -23045,7 +23157,7 @@
         <v>4.4943820224719104</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
         <v>102</v>
       </c>
@@ -23058,7 +23170,7 @@
         <v>3.3707865168539324</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
         <v>108</v>
       </c>
@@ -23080,16 +23192,16 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3A84441-0A46-4810-A40D-2754CCA890ED}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="23" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="23" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>152</v>
       </c>
@@ -23102,7 +23214,7 @@
       </c>
       <c r="E1" s="27"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="17"/>
       <c r="B2" s="17" t="s">
         <v>155</v>
@@ -23117,7 +23229,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>157</v>
       </c>
@@ -23135,7 +23247,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>158</v>
       </c>
@@ -23153,7 +23265,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>159</v>
       </c>
@@ -23171,7 +23283,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>160</v>
       </c>
@@ -23189,7 +23301,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>161</v>
       </c>
@@ -23207,7 +23319,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
         <v>152</v>
       </c>
@@ -23220,7 +23332,7 @@
       </c>
       <c r="E9" s="27"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="17"/>
       <c r="B10" s="17" t="s">
         <v>155</v>
@@ -23235,7 +23347,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>157</v>
       </c>
@@ -23255,7 +23367,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>158</v>
       </c>
@@ -23275,7 +23387,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>159</v>
       </c>
@@ -23295,7 +23407,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>160</v>
       </c>
@@ -23315,7 +23427,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>161</v>
       </c>
@@ -23349,14 +23461,14 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{068D76E6-F265-420D-A051-20972C028530}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>163</v>
       </c>
@@ -23367,7 +23479,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>165</v>
       </c>
@@ -23379,7 +23491,7 @@
         <v>71.910112359550567</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>166</v>
       </c>
@@ -23391,7 +23503,7 @@
         <v>22.471910112359549</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>167</v>
       </c>
@@ -23403,7 +23515,7 @@
         <v>5.6179775280898872</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>12</v>
       </c>
@@ -23424,12 +23536,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>25</v>
       </c>
@@ -23437,7 +23549,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="9">
         <v>2083</v>
       </c>
@@ -23445,7 +23557,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="9">
         <v>2082</v>
       </c>
@@ -23453,7 +23565,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
         <v>2081</v>
       </c>
@@ -23461,7 +23573,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
         <v>2080</v>
       </c>
@@ -23469,7 +23581,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="9">
         <v>2079</v>
       </c>
@@ -23477,7 +23589,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="9">
         <v>2078</v>
       </c>
@@ -23485,7 +23597,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
         <v>2077</v>
       </c>
@@ -23493,7 +23605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
         <v>2076</v>
       </c>
@@ -23501,7 +23613,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
         <v>2075</v>
       </c>
@@ -23509,7 +23621,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
         <v>2074</v>
       </c>
@@ -23517,7 +23629,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>12</v>
       </c>
@@ -23535,9 +23647,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>33</v>
       </c>
@@ -23552,7 +23664,7 @@
       </c>
       <c r="G1" s="27"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="27"/>
       <c r="B2" s="26" t="s">
         <v>36</v>
@@ -23565,7 +23677,7 @@
       <c r="F2" s="27"/>
       <c r="G2" s="27"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="27"/>
       <c r="B3" s="10" t="s">
         <v>37</v>
@@ -23592,7 +23704,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>38</v>
       </c>
@@ -23628,7 +23740,7 @@
         <v>66.875</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>39</v>
       </c>
@@ -23664,7 +23776,7 @@
         <v>33.125</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -23709,13 +23821,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>27</v>
       </c>
@@ -23726,7 +23838,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>30</v>
       </c>
@@ -23745,7 +23857,7 @@
         <v>31.460674157303369</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>31</v>
       </c>
@@ -23764,7 +23876,7 @@
         <v>35.955056179775283</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -23783,7 +23895,7 @@
         <v>25.842696629213485</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>41</v>
       </c>
@@ -23802,7 +23914,7 @@
         <v>6.7415730337078648</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -23825,13 +23937,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17375082-251D-4B38-966E-F88F9E772705}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>42</v>
       </c>
@@ -23842,7 +23954,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>43</v>
       </c>
@@ -23861,7 +23973,7 @@
         <v>67.415730337078656</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>44</v>
       </c>
@@ -23880,7 +23992,7 @@
         <v>25.842696629213485</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>45</v>
       </c>
@@ -23899,7 +24011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>46</v>
       </c>
@@ -23918,7 +24030,7 @@
         <v>6.7415730337078648</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -23941,14 +24053,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313C3968-0C2C-495D-B103-63BB836806C3}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>47</v>
       </c>
@@ -23959,7 +24071,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>49</v>
       </c>
@@ -23972,7 +24084,7 @@
         <v>17.977528089887642</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>50</v>
       </c>
@@ -23985,7 +24097,7 @@
         <v>69.662921348314612</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>51</v>
       </c>
@@ -23997,7 +24109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>52</v>
       </c>
@@ -24009,7 +24121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>32</v>
       </c>
@@ -24021,7 +24133,7 @@
         <v>12.359550561797752</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
         <v>12</v>
       </c>
@@ -24043,14 +24155,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A37B388-6521-440D-9FFB-5546F102E9EC}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>53</v>
       </c>
@@ -24061,7 +24173,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>54</v>
       </c>
@@ -24080,7 +24192,7 @@
         <v>53.932584269662918</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>56</v>
       </c>
@@ -24099,7 +24211,7 @@
         <v>39.325842696629216</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>55</v>
       </c>
@@ -24118,7 +24230,7 @@
         <v>6.7415730337078648</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>12</v>
       </c>
@@ -24140,17 +24252,17 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4681C5CD-AD1E-47C1-9DD5-E5803D1EB1C3}">
   <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
         <v>72</v>
       </c>
@@ -24167,7 +24279,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="27"/>
       <c r="B2" s="9" t="s">
         <v>36</v>
@@ -24184,7 +24296,7 @@
       <c r="F2" s="26"/>
       <c r="G2" s="26"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>57</v>
       </c>
@@ -24214,7 +24326,7 @@
         <v>2.8769707586578628</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
         <v>58</v>
       </c>
@@ -24244,7 +24356,7 @@
         <v>3.1532138525805147</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
         <v>59</v>
       </c>
@@ -24274,7 +24386,7 @@
         <v>7.2210618515024931</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
         <v>60</v>
       </c>
@@ -24304,7 +24416,7 @@
         <v>4.9824821452634414</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
         <v>61</v>
       </c>
@@ -24334,7 +24446,7 @@
         <v>9.4882765125993807</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
         <v>62</v>
       </c>
@@ -24364,7 +24476,7 @@
         <v>8.7168171405470964</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
         <v>63</v>
       </c>
@@ -24394,7 +24506,7 @@
         <v>10.431545613798679</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
         <v>64</v>
       </c>
@@ -24424,7 +24536,7 @@
         <v>8.497843956340116</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
         <v>65</v>
       </c>
@@ -24454,7 +24566,7 @@
         <v>9.7173561514620665</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
         <v>66</v>
       </c>
@@ -24484,7 +24596,7 @@
         <v>7.6876431747742888</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
         <v>67</v>
       </c>
@@ -24514,7 +24626,7 @@
         <v>8.8027220051206037</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>68</v>
       </c>
@@ -24544,7 +24656,7 @@
         <v>8.0784260881282837</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
         <v>69</v>
       </c>
@@ -24574,7 +24686,7 @@
         <v>3.6770650855679827</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>70</v>
       </c>
@@ -24604,7 +24716,7 @@
         <v>6.6685756636571893</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>12</v>
       </c>

</xml_diff>